<commit_message>
fixed salesforce dupes and leads bulk upload
</commit_message>
<xml_diff>
--- a/dummy_salesforce_data.xlsx
+++ b/dummy_salesforce_data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C101"/>
+  <dimension ref="A1:D101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,9 +409,12 @@
       <c r="C1" t="str">
         <v>Status</v>
       </c>
+      <c r="D1" t="str">
+        <v>SO Mobile</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
+      <c r="A2">
         <v>8520147896</v>
       </c>
       <c r="B2" t="str">
@@ -420,9 +423,12 @@
       <c r="C2" t="str">
         <v>Called</v>
       </c>
+      <c r="D2">
+        <v>9000000000</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
+      <c r="A3">
         <v>8521478963</v>
       </c>
       <c r="B3" t="str">
@@ -431,9 +437,12 @@
       <c r="C3" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D3">
+        <v>9000000001</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
+      <c r="A4">
         <v>7412369852</v>
       </c>
       <c r="B4" t="str">
@@ -442,9 +451,12 @@
       <c r="C4" t="str">
         <v>Called</v>
       </c>
+      <c r="D4">
+        <v>9000000002</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="A5">
         <v>7896321445</v>
       </c>
       <c r="B5" t="str">
@@ -453,10 +465,13 @@
       <c r="C5" t="str">
         <v>Called</v>
       </c>
+      <c r="D5">
+        <v>9000000003</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>0987654321</v>
+      <c r="A6">
+        <v>987654321</v>
       </c>
       <c r="B6" t="str">
         <v>Salesforce Eve</v>
@@ -464,9 +479,12 @@
       <c r="C6" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D6">
+        <v>9000000004</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
+      <c r="A7">
         <v>9971101239</v>
       </c>
       <c r="B7" t="str">
@@ -475,9 +493,12 @@
       <c r="C7" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D7">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
+      <c r="A8">
         <v>9507546443</v>
       </c>
       <c r="B8" t="str">
@@ -486,9 +507,12 @@
       <c r="C8" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D8">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
+      <c r="A9">
         <v>9861954719</v>
       </c>
       <c r="B9" t="str">
@@ -497,9 +521,12 @@
       <c r="C9" t="str">
         <v>Called</v>
       </c>
+      <c r="D9">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
+      <c r="A10">
         <v>9531374019</v>
       </c>
       <c r="B10" t="str">
@@ -508,9 +535,12 @@
       <c r="C10" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D10">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
+      <c r="A11">
         <v>9829995365</v>
       </c>
       <c r="B11" t="str">
@@ -519,9 +549,12 @@
       <c r="C11" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D11">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
+      <c r="A12">
         <v>9125434094</v>
       </c>
       <c r="B12" t="str">
@@ -530,9 +563,12 @@
       <c r="C12" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D12">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
+      <c r="A13">
         <v>9765287674</v>
       </c>
       <c r="B13" t="str">
@@ -541,9 +577,12 @@
       <c r="C13" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D13">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="str">
+      <c r="A14">
         <v>9652373189</v>
       </c>
       <c r="B14" t="str">
@@ -552,9 +591,12 @@
       <c r="C14" t="str">
         <v>Called</v>
       </c>
+      <c r="D14">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="str">
+      <c r="A15">
         <v>9445771935</v>
       </c>
       <c r="B15" t="str">
@@ -563,9 +605,12 @@
       <c r="C15" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D15">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="str">
+      <c r="A16">
         <v>9298416430</v>
       </c>
       <c r="B16" t="str">
@@ -574,9 +619,12 @@
       <c r="C16" t="str">
         <v>Called</v>
       </c>
+      <c r="D16">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="str">
+      <c r="A17">
         <v>9728909014</v>
       </c>
       <c r="B17" t="str">
@@ -585,9 +633,12 @@
       <c r="C17" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D17">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="str">
+      <c r="A18">
         <v>9236563115</v>
       </c>
       <c r="B18" t="str">
@@ -596,9 +647,12 @@
       <c r="C18" t="str">
         <v>Called</v>
       </c>
+      <c r="D18">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="str">
+      <c r="A19">
         <v>9415188706</v>
       </c>
       <c r="B19" t="str">
@@ -607,9 +661,12 @@
       <c r="C19" t="str">
         <v>Called</v>
       </c>
+      <c r="D19">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="str">
+      <c r="A20">
         <v>9196618212</v>
       </c>
       <c r="B20" t="str">
@@ -618,9 +675,12 @@
       <c r="C20" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D20">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="str">
+      <c r="A21">
         <v>9565306975</v>
       </c>
       <c r="B21" t="str">
@@ -629,9 +689,12 @@
       <c r="C21" t="str">
         <v>Called</v>
       </c>
+      <c r="D21">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="str">
+      <c r="A22">
         <v>9790247450</v>
       </c>
       <c r="B22" t="str">
@@ -640,9 +703,12 @@
       <c r="C22" t="str">
         <v>Called</v>
       </c>
+      <c r="D22">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" t="str">
+      <c r="A23">
         <v>9821491534</v>
       </c>
       <c r="B23" t="str">
@@ -651,9 +717,12 @@
       <c r="C23" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D23">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="str">
+      <c r="A24">
         <v>9256318289</v>
       </c>
       <c r="B24" t="str">
@@ -662,9 +731,12 @@
       <c r="C24" t="str">
         <v>Called</v>
       </c>
+      <c r="D24">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" t="str">
+      <c r="A25">
         <v>9398518510</v>
       </c>
       <c r="B25" t="str">
@@ -673,9 +745,12 @@
       <c r="C25" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D25">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" t="str">
+      <c r="A26">
         <v>9777317274</v>
       </c>
       <c r="B26" t="str">
@@ -684,9 +759,12 @@
       <c r="C26" t="str">
         <v>Called</v>
       </c>
+      <c r="D26">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" t="str">
+      <c r="A27">
         <v>9480228816</v>
       </c>
       <c r="B27" t="str">
@@ -695,9 +773,12 @@
       <c r="C27" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D27">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" t="str">
+      <c r="A28">
         <v>9962685133</v>
       </c>
       <c r="B28" t="str">
@@ -706,9 +787,12 @@
       <c r="C28" t="str">
         <v>Called</v>
       </c>
+      <c r="D28">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" t="str">
+      <c r="A29">
         <v>9374477004</v>
       </c>
       <c r="B29" t="str">
@@ -717,9 +801,12 @@
       <c r="C29" t="str">
         <v>Called</v>
       </c>
+      <c r="D29">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="str">
+      <c r="A30">
         <v>9216116552</v>
       </c>
       <c r="B30" t="str">
@@ -728,9 +815,12 @@
       <c r="C30" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D30">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" t="str">
+      <c r="A31">
         <v>9444514383</v>
       </c>
       <c r="B31" t="str">
@@ -739,9 +829,12 @@
       <c r="C31" t="str">
         <v>Called</v>
       </c>
+      <c r="D31">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" t="str">
+      <c r="A32">
         <v>9480383131</v>
       </c>
       <c r="B32" t="str">
@@ -750,9 +843,12 @@
       <c r="C32" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D32">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" t="str">
+      <c r="A33">
         <v>9679071348</v>
       </c>
       <c r="B33" t="str">
@@ -761,9 +857,12 @@
       <c r="C33" t="str">
         <v>Called</v>
       </c>
+      <c r="D33">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" t="str">
+      <c r="A34">
         <v>9640142894</v>
       </c>
       <c r="B34" t="str">
@@ -772,9 +871,12 @@
       <c r="C34" t="str">
         <v>Called</v>
       </c>
+      <c r="D34">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" t="str">
+      <c r="A35">
         <v>9501769607</v>
       </c>
       <c r="B35" t="str">
@@ -783,9 +885,12 @@
       <c r="C35" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D35">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" t="str">
+      <c r="A36">
         <v>9872469079</v>
       </c>
       <c r="B36" t="str">
@@ -794,9 +899,12 @@
       <c r="C36" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D36">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" t="str">
+      <c r="A37">
         <v>9179289566</v>
       </c>
       <c r="B37" t="str">
@@ -805,9 +913,12 @@
       <c r="C37" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D37">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" t="str">
+      <c r="A38">
         <v>9721957559</v>
       </c>
       <c r="B38" t="str">
@@ -816,9 +927,12 @@
       <c r="C38" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D38">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" t="str">
+      <c r="A39">
         <v>9909376873</v>
       </c>
       <c r="B39" t="str">
@@ -827,9 +941,12 @@
       <c r="C39" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D39">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" t="str">
+      <c r="A40">
         <v>9259629009</v>
       </c>
       <c r="B40" t="str">
@@ -838,9 +955,12 @@
       <c r="C40" t="str">
         <v>Called</v>
       </c>
+      <c r="D40">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" t="str">
+      <c r="A41">
         <v>9579544585</v>
       </c>
       <c r="B41" t="str">
@@ -849,9 +969,12 @@
       <c r="C41" t="str">
         <v>Called</v>
       </c>
+      <c r="D41">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" t="str">
+      <c r="A42">
         <v>9100796571</v>
       </c>
       <c r="B42" t="str">
@@ -860,9 +983,12 @@
       <c r="C42" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D42">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" t="str">
+      <c r="A43">
         <v>9680802175</v>
       </c>
       <c r="B43" t="str">
@@ -871,9 +997,12 @@
       <c r="C43" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D43">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" t="str">
+      <c r="A44">
         <v>9568216541</v>
       </c>
       <c r="B44" t="str">
@@ -882,9 +1011,12 @@
       <c r="C44" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D44">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" t="str">
+      <c r="A45">
         <v>9538618219</v>
       </c>
       <c r="B45" t="str">
@@ -893,9 +1025,12 @@
       <c r="C45" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D45">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" t="str">
+      <c r="A46">
         <v>9712713448</v>
       </c>
       <c r="B46" t="str">
@@ -904,9 +1039,12 @@
       <c r="C46" t="str">
         <v>Called</v>
       </c>
+      <c r="D46">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" t="str">
+      <c r="A47">
         <v>9993757478</v>
       </c>
       <c r="B47" t="str">
@@ -915,9 +1053,12 @@
       <c r="C47" t="str">
         <v>Called</v>
       </c>
+      <c r="D47">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" t="str">
+      <c r="A48">
         <v>9382164516</v>
       </c>
       <c r="B48" t="str">
@@ -926,9 +1067,12 @@
       <c r="C48" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D48">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="str">
+      <c r="A49">
         <v>9769763569</v>
       </c>
       <c r="B49" t="str">
@@ -937,9 +1081,12 @@
       <c r="C49" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D49">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" t="str">
+      <c r="A50">
         <v>9255545026</v>
       </c>
       <c r="B50" t="str">
@@ -948,9 +1095,12 @@
       <c r="C50" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D50">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" t="str">
+      <c r="A51">
         <v>9492193566</v>
       </c>
       <c r="B51" t="str">
@@ -959,9 +1109,12 @@
       <c r="C51" t="str">
         <v>Called</v>
       </c>
+      <c r="D51">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" t="str">
+      <c r="A52">
         <v>9100527933</v>
       </c>
       <c r="B52" t="str">
@@ -970,9 +1123,12 @@
       <c r="C52" t="str">
         <v>Called</v>
       </c>
+      <c r="D52">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" t="str">
+      <c r="A53">
         <v>9421082626</v>
       </c>
       <c r="B53" t="str">
@@ -981,9 +1137,12 @@
       <c r="C53" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D53">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" t="str">
+      <c r="A54">
         <v>9175597054</v>
       </c>
       <c r="B54" t="str">
@@ -992,9 +1151,12 @@
       <c r="C54" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D54">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" t="str">
+      <c r="A55">
         <v>9779796362</v>
       </c>
       <c r="B55" t="str">
@@ -1003,9 +1165,12 @@
       <c r="C55" t="str">
         <v>Called</v>
       </c>
+      <c r="D55">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" t="str">
+      <c r="A56">
         <v>9938695736</v>
       </c>
       <c r="B56" t="str">
@@ -1014,9 +1179,12 @@
       <c r="C56" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D56">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" t="str">
+      <c r="A57">
         <v>9110718949</v>
       </c>
       <c r="B57" t="str">
@@ -1025,9 +1193,12 @@
       <c r="C57" t="str">
         <v>Called</v>
       </c>
+      <c r="D57">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" t="str">
+      <c r="A58">
         <v>9490481581</v>
       </c>
       <c r="B58" t="str">
@@ -1036,9 +1207,12 @@
       <c r="C58" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D58">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" t="str">
+      <c r="A59">
         <v>9209553505</v>
       </c>
       <c r="B59" t="str">
@@ -1047,9 +1221,12 @@
       <c r="C59" t="str">
         <v>Called</v>
       </c>
+      <c r="D59">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" t="str">
+      <c r="A60">
         <v>9708008265</v>
       </c>
       <c r="B60" t="str">
@@ -1058,9 +1235,12 @@
       <c r="C60" t="str">
         <v>Called</v>
       </c>
+      <c r="D60">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" t="str">
+      <c r="A61">
         <v>9417041775</v>
       </c>
       <c r="B61" t="str">
@@ -1069,9 +1249,12 @@
       <c r="C61" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D61">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" t="str">
+      <c r="A62">
         <v>9129482525</v>
       </c>
       <c r="B62" t="str">
@@ -1080,9 +1263,12 @@
       <c r="C62" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D62">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" t="str">
+      <c r="A63">
         <v>9541716510</v>
       </c>
       <c r="B63" t="str">
@@ -1091,9 +1277,12 @@
       <c r="C63" t="str">
         <v>Called</v>
       </c>
+      <c r="D63">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" t="str">
+      <c r="A64">
         <v>9770234586</v>
       </c>
       <c r="B64" t="str">
@@ -1102,9 +1291,12 @@
       <c r="C64" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D64">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" t="str">
+      <c r="A65">
         <v>9468013995</v>
       </c>
       <c r="B65" t="str">
@@ -1113,9 +1305,12 @@
       <c r="C65" t="str">
         <v>Called</v>
       </c>
+      <c r="D65">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" t="str">
+      <c r="A66">
         <v>9364217156</v>
       </c>
       <c r="B66" t="str">
@@ -1124,9 +1319,12 @@
       <c r="C66" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D66">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" t="str">
+      <c r="A67">
         <v>9578967437</v>
       </c>
       <c r="B67" t="str">
@@ -1135,9 +1333,12 @@
       <c r="C67" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D67">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" t="str">
+      <c r="A68">
         <v>9735532983</v>
       </c>
       <c r="B68" t="str">
@@ -1146,9 +1347,12 @@
       <c r="C68" t="str">
         <v>Called</v>
       </c>
+      <c r="D68">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" t="str">
+      <c r="A69">
         <v>9839859588</v>
       </c>
       <c r="B69" t="str">
@@ -1157,9 +1361,12 @@
       <c r="C69" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D69">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" t="str">
+      <c r="A70">
         <v>9318124521</v>
       </c>
       <c r="B70" t="str">
@@ -1168,9 +1375,12 @@
       <c r="C70" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D70">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" t="str">
+      <c r="A71">
         <v>9456050652</v>
       </c>
       <c r="B71" t="str">
@@ -1179,9 +1389,12 @@
       <c r="C71" t="str">
         <v>Called</v>
       </c>
+      <c r="D71">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" t="str">
+      <c r="A72">
         <v>9400507076</v>
       </c>
       <c r="B72" t="str">
@@ -1190,9 +1403,12 @@
       <c r="C72" t="str">
         <v>Called</v>
       </c>
+      <c r="D72">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" t="str">
+      <c r="A73">
         <v>9850139505</v>
       </c>
       <c r="B73" t="str">
@@ -1201,9 +1417,12 @@
       <c r="C73" t="str">
         <v>Called</v>
       </c>
+      <c r="D73">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" t="str">
+      <c r="A74">
         <v>9465478758</v>
       </c>
       <c r="B74" t="str">
@@ -1212,9 +1431,12 @@
       <c r="C74" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D74">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" t="str">
+      <c r="A75">
         <v>9435762828</v>
       </c>
       <c r="B75" t="str">
@@ -1223,9 +1445,12 @@
       <c r="C75" t="str">
         <v>Called</v>
       </c>
+      <c r="D75">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" t="str">
+      <c r="A76">
         <v>9807745784</v>
       </c>
       <c r="B76" t="str">
@@ -1234,9 +1459,12 @@
       <c r="C76" t="str">
         <v>Called</v>
       </c>
+      <c r="D76">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" t="str">
+      <c r="A77">
         <v>9501570101</v>
       </c>
       <c r="B77" t="str">
@@ -1245,9 +1473,12 @@
       <c r="C77" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D77">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" t="str">
+      <c r="A78">
         <v>9293438218</v>
       </c>
       <c r="B78" t="str">
@@ -1256,9 +1487,12 @@
       <c r="C78" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D78">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" t="str">
+      <c r="A79">
         <v>9707437080</v>
       </c>
       <c r="B79" t="str">
@@ -1267,9 +1501,12 @@
       <c r="C79" t="str">
         <v>Called</v>
       </c>
+      <c r="D79">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" t="str">
+      <c r="A80">
         <v>9900924400</v>
       </c>
       <c r="B80" t="str">
@@ -1278,9 +1515,12 @@
       <c r="C80" t="str">
         <v>Called</v>
       </c>
+      <c r="D80">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" t="str">
+      <c r="A81">
         <v>9260778967</v>
       </c>
       <c r="B81" t="str">
@@ -1289,9 +1529,12 @@
       <c r="C81" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D81">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" t="str">
+      <c r="A82">
         <v>9725809910</v>
       </c>
       <c r="B82" t="str">
@@ -1300,9 +1543,12 @@
       <c r="C82" t="str">
         <v>Called</v>
       </c>
+      <c r="D82">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" t="str">
+      <c r="A83">
         <v>9880530607</v>
       </c>
       <c r="B83" t="str">
@@ -1311,9 +1557,12 @@
       <c r="C83" t="str">
         <v>Called</v>
       </c>
+      <c r="D83">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" t="str">
+      <c r="A84">
         <v>9803013822</v>
       </c>
       <c r="B84" t="str">
@@ -1322,9 +1571,12 @@
       <c r="C84" t="str">
         <v>Called</v>
       </c>
+      <c r="D84">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" t="str">
+      <c r="A85">
         <v>9552816463</v>
       </c>
       <c r="B85" t="str">
@@ -1333,9 +1585,12 @@
       <c r="C85" t="str">
         <v>Called</v>
       </c>
+      <c r="D85">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" t="str">
+      <c r="A86">
         <v>9584194162</v>
       </c>
       <c r="B86" t="str">
@@ -1344,9 +1599,12 @@
       <c r="C86" t="str">
         <v>Called</v>
       </c>
+      <c r="D86">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" t="str">
+      <c r="A87">
         <v>9327292914</v>
       </c>
       <c r="B87" t="str">
@@ -1355,9 +1613,12 @@
       <c r="C87" t="str">
         <v>Called</v>
       </c>
+      <c r="D87">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" t="str">
+      <c r="A88">
         <v>9691140517</v>
       </c>
       <c r="B88" t="str">
@@ -1366,9 +1627,12 @@
       <c r="C88" t="str">
         <v>Called</v>
       </c>
+      <c r="D88">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" t="str">
+      <c r="A89">
         <v>9902590827</v>
       </c>
       <c r="B89" t="str">
@@ -1377,9 +1641,12 @@
       <c r="C89" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D89">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" t="str">
+      <c r="A90">
         <v>9987951394</v>
       </c>
       <c r="B90" t="str">
@@ -1388,9 +1655,12 @@
       <c r="C90" t="str">
         <v>Called</v>
       </c>
+      <c r="D90">
+        <v>9000000008</v>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" t="str">
+      <c r="A91">
         <v>9234058959</v>
       </c>
       <c r="B91" t="str">
@@ -1399,9 +1669,12 @@
       <c r="C91" t="str">
         <v>Called</v>
       </c>
+      <c r="D91">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="92">
-      <c r="A92" t="str">
+      <c r="A92">
         <v>9811918483</v>
       </c>
       <c r="B92" t="str">
@@ -1410,9 +1683,12 @@
       <c r="C92" t="str">
         <v>Called</v>
       </c>
+      <c r="D92">
+        <v>9000000007</v>
+      </c>
     </row>
     <row r="93">
-      <c r="A93" t="str">
+      <c r="A93">
         <v>9607743392</v>
       </c>
       <c r="B93" t="str">
@@ -1421,9 +1697,12 @@
       <c r="C93" t="str">
         <v>Called</v>
       </c>
+      <c r="D93">
+        <v>9000000010</v>
+      </c>
     </row>
     <row r="94">
-      <c r="A94" t="str">
+      <c r="A94">
         <v>9709392826</v>
       </c>
       <c r="B94" t="str">
@@ -1432,9 +1711,12 @@
       <c r="C94" t="str">
         <v>Called</v>
       </c>
+      <c r="D94">
+        <v>9000000009</v>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" t="str">
+      <c r="A95">
         <v>9289184327</v>
       </c>
       <c r="B95" t="str">
@@ -1443,9 +1725,12 @@
       <c r="C95" t="str">
         <v>Called</v>
       </c>
+      <c r="D95">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="96">
-      <c r="A96" t="str">
+      <c r="A96">
         <v>9577362803</v>
       </c>
       <c r="B96" t="str">
@@ -1454,9 +1739,12 @@
       <c r="C96" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D96">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" t="str">
+      <c r="A97">
         <v>9815256724</v>
       </c>
       <c r="B97" t="str">
@@ -1465,9 +1753,12 @@
       <c r="C97" t="str">
         <v>Called</v>
       </c>
+      <c r="D97">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" t="str">
+      <c r="A98">
         <v>9236305245</v>
       </c>
       <c r="B98" t="str">
@@ -1476,9 +1767,12 @@
       <c r="C98" t="str">
         <v>Called</v>
       </c>
+      <c r="D98">
+        <v>9000000006</v>
+      </c>
     </row>
     <row r="99">
-      <c r="A99" t="str">
+      <c r="A99">
         <v>9855255507</v>
       </c>
       <c r="B99" t="str">
@@ -1487,9 +1781,12 @@
       <c r="C99" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D99">
+        <v>9000000011</v>
+      </c>
     </row>
     <row r="100">
-      <c r="A100" t="str">
+      <c r="A100">
         <v>9899773026</v>
       </c>
       <c r="B100" t="str">
@@ -1498,9 +1795,12 @@
       <c r="C100" t="str">
         <v>Called</v>
       </c>
+      <c r="D100">
+        <v>9000000005</v>
+      </c>
     </row>
     <row r="101">
-      <c r="A101" t="str">
+      <c r="A101">
         <v>9905564690</v>
       </c>
       <c r="B101" t="str">
@@ -1509,10 +1809,13 @@
       <c r="C101" t="str">
         <v>Not Reachable</v>
       </c>
+      <c r="D101">
+        <v>9000000010</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>